<commit_message>
Give railgun a table-driven 3.5s main-cannon cadence and bounded warm effects
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/weapon_motion.xlsx
+++ b/space-battleship/config_excel/weapon_motion.xlsx
@@ -1207,7 +1207,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="3" width="30" customWidth="1"/>
@@ -1622,6 +1622,206 @@
         <v>30</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>rail_charge_seconds</t>
+        </is>
+      </c>
+      <c r="B25" s="0">
+        <v>0.9</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>游戏秒</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>玩家磁轨炮周期末段蓄力表现；包含在equipment.cannon.cd内，随合法冷却倍率同比缩放</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t>玩家磁轨炮表现</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>rail_charge_radius</t>
+        </is>
+      </c>
+      <c r="B26" s="0">
+        <v>20</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>显示像素</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>局部炮口蓄力环半径</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>玩家磁轨炮表现</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>rail_trail_length</t>
+        </is>
+      </c>
+      <c r="B27" s="0">
+        <v>138</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>显示像素</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>磁轨弹头后方短弹道最大长度；不连接整条炮口到目标</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t>玩家磁轨炮表现</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>rail_trail_width</t>
+        </is>
+      </c>
+      <c r="B28" s="0">
+        <v>10</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>显示像素</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>磁轨主炮弹道宽度</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>玩家磁轨炮表现</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>rail_flash_seconds</t>
+        </is>
+      </c>
+      <c r="B29" s="0">
+        <v>0.09</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>显示秒</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>主炮局部炮口闪光时长</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t>玩家磁轨炮表现</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>rail_impact_seconds</t>
+        </is>
+      </c>
+      <c r="B30" s="0">
+        <v>0.16</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>显示秒</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>主炮局部命中冲击时长</t>
+        </is>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t>玩家磁轨炮表现</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>rail_impact_radius</t>
+        </is>
+      </c>
+      <c r="B31" s="0">
+        <v>24</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>显示像素</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>主炮命中冲击半径</t>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t>玩家磁轨炮表现</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>rail_penetration_length</t>
+        </is>
+      </c>
+      <c r="B32" s="0">
+        <v>80</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>显示像素</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>命中处向前的短促视觉冲击长度；不改变命中与连锁</t>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t>玩家磁轨炮表现</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A3:E24" etc:filterBottomFollowUsedRange="0">
     <extLst/>

</xml_diff>

<commit_message>
Broaden railgun body and make presentation regression table-aware
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/weapon_motion.xlsx
+++ b/space-battleship/config_excel/weapon_motion.xlsx
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="B26" s="0">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
       <c r="B28" s="0">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="B31" s="0">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>

</xml_diff>